<commit_message>
i4 write to data class from xl
</commit_message>
<xml_diff>
--- a/Indicator_4/Real_data/Bigeye_Tuna_Atl.xlsx
+++ b/Indicator_4/Real_data/Bigeye_Tuna_Atl.xlsx
@@ -1,22 +1,300 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\EcoTest_Train\Indicator_4\Real_data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{325AB6B7-2AC0-42AA-A7BA-1A7376D09756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
     <sheet name="Time_series" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="89">
+  <si>
+    <t>Parameter</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Bigeye_Tuna_Atl</t>
+  </si>
+  <si>
+    <t>E.g. 'Swordfish_Natl'</t>
+  </si>
+  <si>
+    <t>Stock</t>
+  </si>
+  <si>
+    <t>max_age</t>
+  </si>
+  <si>
+    <t>5.65</t>
+  </si>
+  <si>
+    <t>Age to 5% natural survival</t>
+  </si>
+  <si>
+    <t>Life history</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>0.42</t>
+  </si>
+  <si>
+    <t>von Bertalannfy K</t>
+  </si>
+  <si>
+    <t>Linf</t>
+  </si>
+  <si>
+    <t>0.588</t>
+  </si>
+  <si>
+    <t>von Bertalannfy L-infinity (asymptotic length)</t>
+  </si>
+  <si>
+    <t>L50_Linf</t>
+  </si>
+  <si>
+    <t>178.6</t>
+  </si>
+  <si>
+    <t>Length at 50% maturity relative to asymptotic length (von B. L-infinity)</t>
+  </si>
+  <si>
+    <t>Total_L5_L50</t>
+  </si>
+  <si>
+    <t>0.318</t>
+  </si>
+  <si>
+    <t>Length at 5% selection relative to length at 50% maturity</t>
+  </si>
+  <si>
+    <t>Fleet selectivity</t>
+  </si>
+  <si>
+    <t>All fleets combined</t>
+  </si>
+  <si>
+    <t>Total_LFS_L50</t>
+  </si>
+  <si>
+    <t>1.224</t>
+  </si>
+  <si>
+    <t>Length at full selection relative to length at 50% maturity</t>
+  </si>
+  <si>
+    <t>Total_VML</t>
+  </si>
+  <si>
+    <t>0.408</t>
+  </si>
+  <si>
+    <t>Selectivity of maximum length class</t>
+  </si>
+  <si>
+    <t>Fleet_1_L5_L50</t>
+  </si>
+  <si>
+    <t>0.756</t>
+  </si>
+  <si>
+    <t>Fleet 1</t>
+  </si>
+  <si>
+    <t>Fleet_1_LFS_L50</t>
+  </si>
+  <si>
+    <t>1.182</t>
+  </si>
+  <si>
+    <t>Fleet_1_VML</t>
+  </si>
+  <si>
+    <t>0.007</t>
+  </si>
+  <si>
+    <t>Fleet_2_L5_L50</t>
+  </si>
+  <si>
+    <t>0.303</t>
+  </si>
+  <si>
+    <t>Fleet 2</t>
+  </si>
+  <si>
+    <t>Fleet_2_LFS_L50</t>
+  </si>
+  <si>
+    <t>0.433</t>
+  </si>
+  <si>
+    <t>Fleet_2_VML</t>
+  </si>
+  <si>
+    <t>0.008</t>
+  </si>
+  <si>
+    <t>Fleet_3_L5_L50</t>
+  </si>
+  <si>
+    <t>0.378</t>
+  </si>
+  <si>
+    <t>Fleet 3</t>
+  </si>
+  <si>
+    <t>Fleet_3_LFS_L50</t>
+  </si>
+  <si>
+    <t>1.233</t>
+  </si>
+  <si>
+    <t>Fleet_3_VML</t>
+  </si>
+  <si>
+    <t>0.512</t>
+  </si>
+  <si>
+    <t>Fleet_1_CF</t>
+  </si>
+  <si>
+    <t>0.179</t>
+  </si>
+  <si>
+    <t>Fraction of all historical catches that were Fleet 1</t>
+  </si>
+  <si>
+    <t>Fleet catch scale</t>
+  </si>
+  <si>
+    <t>Fleet_2_CF</t>
+  </si>
+  <si>
+    <t>0.107</t>
+  </si>
+  <si>
+    <t>Fraction of all historical catches that were Fleet 2</t>
+  </si>
+  <si>
+    <t>Fleet_3_CF</t>
+  </si>
+  <si>
+    <t>0.714</t>
+  </si>
+  <si>
+    <t>Fraction of all historical catches that were Fleet 3</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Total_catch</t>
+  </si>
+  <si>
+    <t>Total_mean_len</t>
+  </si>
+  <si>
+    <t>Total_mean_age</t>
+  </si>
+  <si>
+    <t>Total_CV_len</t>
+  </si>
+  <si>
+    <t>Total_frac_mat</t>
+  </si>
+  <si>
+    <t>Total_Index</t>
+  </si>
+  <si>
+    <t>Fleet_1_catch</t>
+  </si>
+  <si>
+    <t>Fleet_1_mean_len</t>
+  </si>
+  <si>
+    <t>Fleet_1_mean_age</t>
+  </si>
+  <si>
+    <t>Fleet_1_CV_len</t>
+  </si>
+  <si>
+    <t>Fleet_1_frac_mat</t>
+  </si>
+  <si>
+    <t>Fleet_1_Index</t>
+  </si>
+  <si>
+    <t>Fleet_2_catch</t>
+  </si>
+  <si>
+    <t>Fleet_2_mean_len</t>
+  </si>
+  <si>
+    <t>Fleet_2_mean_age</t>
+  </si>
+  <si>
+    <t>Fleet_2_CV_len</t>
+  </si>
+  <si>
+    <t>Fleet_2_frac_mat</t>
+  </si>
+  <si>
+    <t>Fleet_2_Index</t>
+  </si>
+  <si>
+    <t>Fleet_3_catch</t>
+  </si>
+  <si>
+    <t>Fleet_3_mean_len</t>
+  </si>
+  <si>
+    <t>Fleet_3_mean_age</t>
+  </si>
+  <si>
+    <t>Fleet_3_CV_len</t>
+  </si>
+  <si>
+    <t>Fleet_3_frac_mat</t>
+  </si>
+  <si>
+    <t>Fleet_3_Index</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -64,13 +342,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -108,7 +394,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -142,6 +428,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -176,9 +463,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -351,656 +639,368 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Parameter</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Bigeye_Tuna_Atl</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Genus specius</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Billfish</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>North Atlantic</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>max_age</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>5.65</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Age to 5% natural survival</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Life history</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>0.42</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>von Bertalannfy K</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Life history</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>L50_Linf</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>0.588</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Length at 50% maturity relative to asymptotic length (von B. L-infinity)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Life history</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Stock</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>All_L5_L50</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>0.318</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Length at 5% selection relative to length at 50% maturity</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>All fleets combined</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>All_LFS_L50</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1.224</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Length at full selection relative to length at 50% maturity</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>All fleets combined</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>All_VML</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>0.408</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Selectivity of maximum length class</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>All fleets combined</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Fleet_1_L5_L50</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>0.756</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Length at 5% selection relative to length at 50% maturity</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Fleet 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Fleet_1_LFS_L50</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>1.182</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Length at full selection relative to length at 50% maturity</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Fleet 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Fleet_1_VML</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>0.007</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Selectivity of maximum length class</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Fleet 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Fleet_2_L5_L50</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>0.303</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Length at 5% selection relative to length at 50% maturity</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Fleet 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Fleet_2_LFS_L50</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>0.433</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Length at full selection relative to length at 50% maturity</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Fleet 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Fleet_2_VML</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>0.008</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Selectivity of maximum length class</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Fleet 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Fleet_3_L5_L50</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>0.378</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Length at 5% selection relative to length at 50% maturity</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Fleet 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Fleet_3_LFS_L50</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>1.233</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Length at full selection relative to length at 50% maturity</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Fleet 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Fleet_3_VML</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>0.512</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Selectivity of maximum length class</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Fleet selectivity</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Fleet 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>All_ML_Linf</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>0.614</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Last historical mean length relative to Linf (e.g. mulen(2024) / Linf)</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Fleet catch-length</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>All fleets combined</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Fleet_1_ML_Linf</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>0.723</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Last historical mean length relative to Linf (e.g. mulen(2024) / Linf)</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Fleet catch-length</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Fleet 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Fleet_2_ML_Linf</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>0.286</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Last historical mean length relative to Linf (e.g. mulen(2024) / Linf)</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Fleet catch-length</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Fleet 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Fleet_3_ML_Linf</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>0.621</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Last historical mean length relative to Linf (e.g. mulen(2024) / Linf)</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Fleet catch-length</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Fleet 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Fleet_1_CF</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>0.179</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Fraction of all historical catches that were Fleet 1</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Fleet catch scale</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Fleet 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Fleet_2_CF</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>0.107</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Fraction of all historical catches that were Fleet 2</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Fleet catch scale</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Fleet 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Fleet_3_CF</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>0.714</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Fraction of all historical catches that were Fleet 3</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Fleet catch scale</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Fleet 3</t>
-        </is>
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1009,138 +1009,88 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Y71"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Total_catch</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Total_mean_len</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Total_mean_age</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Total_CV_len</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Total_frac_mat</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Total_Index</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_1_catch</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_1_mean_len</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_1_mean_age</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_1_CV_len</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_1_frac_mat</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_1_Index</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_2_catch</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_2_mean_len</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_2_mean_age</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_2_CV_len</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_2_frac_mat</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_2_Index</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_3_catch</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_3_mean_len</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_3_mean_age</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_3_CV_len</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_3_frac_mat</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Fleet_3_Index</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+    <row r="1" spans="1:25" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1950</v>
       </c>
@@ -1157,7 +1107,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1951</v>
       </c>
@@ -1174,7 +1124,7 @@
         <v>1651</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1952</v>
       </c>
@@ -1191,7 +1141,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1953</v>
       </c>
@@ -1208,7 +1158,7 @@
         <v>2951</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1954</v>
       </c>
@@ -1225,7 +1175,7 @@
         <v>2932</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1955</v>
       </c>
@@ -1242,7 +1192,7 @@
         <v>4808</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1956</v>
       </c>
@@ -1259,7 +1209,7 @@
         <v>2769</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1957</v>
       </c>
@@ -1276,7 +1226,7 @@
         <v>8266.1</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1958</v>
       </c>
@@ -1293,7 +1243,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1959</v>
       </c>
@@ -1304,7 +1254,7 @@
         <v>1443.4</v>
       </c>
       <c r="M11">
-        <v>0.854</v>
+        <v>0.85399999999999998</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -1313,7 +1263,7 @@
         <v>6288.6</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1960</v>
       </c>
@@ -1324,7 +1274,7 @@
         <v>2750.8</v>
       </c>
       <c r="M12">
-        <v>0.9360000000000001</v>
+        <v>0.93600000000000005</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -1333,7 +1283,7 @@
         <v>6362.1</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1961</v>
       </c>
@@ -1353,7 +1303,7 @@
         <v>11304.8</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1962</v>
       </c>
@@ -1364,7 +1314,7 @@
         <v>12667.7</v>
       </c>
       <c r="M14">
-        <v>1.017</v>
+        <v>1.0169999999999999</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -1373,7 +1323,7 @@
         <v>10464.1</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1963</v>
       </c>
@@ -1393,7 +1343,7 @@
         <v>15682.6</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1964</v>
       </c>
@@ -1413,12 +1363,12 @@
         <v>10387.9</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1965</v>
       </c>
       <c r="B17">
-        <v>39393.8</v>
+        <v>39393.800000000003</v>
       </c>
       <c r="C17">
         <v>131.72</v>
@@ -1427,19 +1377,19 @@
         <v>0.872</v>
       </c>
       <c r="H17">
-        <v>16880.9</v>
+        <v>16880.900000000001</v>
       </c>
       <c r="I17">
         <v>136.751</v>
       </c>
       <c r="K17">
-        <v>0.165</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="L17">
         <v>0.876</v>
       </c>
       <c r="M17">
-        <v>1.251</v>
+        <v>1.2509999999999999</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -1448,27 +1398,27 @@
         <v>22512.9</v>
       </c>
       <c r="U17">
-        <v>129.205</v>
+        <v>129.20500000000001</v>
       </c>
       <c r="X17">
-        <v>0.869</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>0.86899999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1966</v>
       </c>
       <c r="B18">
-        <v>25386.4</v>
+        <v>25386.400000000001</v>
       </c>
       <c r="C18">
         <v>124.746</v>
       </c>
       <c r="E18">
-        <v>0.206</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="F18">
-        <v>0.772</v>
+        <v>0.77200000000000002</v>
       </c>
       <c r="H18">
         <v>11158.7</v>
@@ -1480,10 +1430,10 @@
         <v>0.189</v>
       </c>
       <c r="L18">
-        <v>0.766</v>
+        <v>0.76600000000000001</v>
       </c>
       <c r="M18">
-        <v>1.098</v>
+        <v>1.0980000000000001</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -1498,10 +1448,10 @@
         <v>0.22</v>
       </c>
       <c r="X18">
-        <v>0.776</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>0.77600000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1967</v>
       </c>
@@ -1521,16 +1471,16 @@
         <v>5842</v>
       </c>
       <c r="I19">
-        <v>130.808</v>
+        <v>130.80799999999999</v>
       </c>
       <c r="K19">
         <v>0.158</v>
       </c>
       <c r="L19">
-        <v>0.862</v>
+        <v>0.86199999999999999</v>
       </c>
       <c r="M19">
-        <v>1.058</v>
+        <v>1.0580000000000001</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -1539,7 +1489,7 @@
         <v>19410.2</v>
       </c>
       <c r="U19">
-        <v>106.019</v>
+        <v>106.01900000000001</v>
       </c>
       <c r="W19">
         <v>0.245</v>
@@ -1548,33 +1498,33 @@
         <v>0.499</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>1968</v>
       </c>
       <c r="B20">
-        <v>23911.2</v>
+        <v>23911.200000000001</v>
       </c>
       <c r="C20">
         <v>121.185</v>
       </c>
       <c r="E20">
-        <v>0.199</v>
+        <v>0.19900000000000001</v>
       </c>
       <c r="F20">
-        <v>0.728</v>
+        <v>0.72799999999999998</v>
       </c>
       <c r="H20">
         <v>4079.9</v>
       </c>
       <c r="I20">
-        <v>128.907</v>
+        <v>128.90700000000001</v>
       </c>
       <c r="K20">
         <v>0.193</v>
       </c>
       <c r="L20">
-        <v>0.823</v>
+        <v>0.82299999999999995</v>
       </c>
       <c r="M20">
         <v>1.21</v>
@@ -1586,16 +1536,16 @@
         <v>19831.3</v>
       </c>
       <c r="U20">
-        <v>115.007</v>
+        <v>115.00700000000001</v>
       </c>
       <c r="W20">
-        <v>0.204</v>
+        <v>0.20399999999999999</v>
       </c>
       <c r="X20">
-        <v>0.652</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>0.65200000000000002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>1969</v>
       </c>
@@ -1609,7 +1559,7 @@
         <v>0.218</v>
       </c>
       <c r="F21">
-        <v>0.643</v>
+        <v>0.64300000000000002</v>
       </c>
       <c r="H21">
         <v>3137.7</v>
@@ -1618,42 +1568,42 @@
         <v>117.69</v>
       </c>
       <c r="K21">
-        <v>0.198</v>
+        <v>0.19800000000000001</v>
       </c>
       <c r="L21">
-        <v>0.592</v>
+        <v>0.59199999999999997</v>
       </c>
       <c r="M21">
-        <v>1.088</v>
+        <v>1.0880000000000001</v>
       </c>
       <c r="N21">
         <v>0</v>
       </c>
       <c r="T21">
-        <v>33597.8</v>
+        <v>33597.800000000003</v>
       </c>
       <c r="U21">
         <v>122.19</v>
       </c>
       <c r="W21">
-        <v>0.231</v>
+        <v>0.23100000000000001</v>
       </c>
       <c r="X21">
-        <v>0.674</v>
-      </c>
-    </row>
-    <row r="22">
+        <v>0.67400000000000004</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>1970</v>
       </c>
       <c r="B22">
-        <v>41879.7</v>
+        <v>41879.699999999997</v>
       </c>
       <c r="C22">
-        <v>128.842</v>
+        <v>128.84200000000001</v>
       </c>
       <c r="E22">
-        <v>0.164</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="F22">
         <v>0.83</v>
@@ -1662,16 +1612,16 @@
         <v>3609.6</v>
       </c>
       <c r="I22">
-        <v>128.207</v>
+        <v>128.20699999999999</v>
       </c>
       <c r="K22">
-        <v>0.179</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="L22">
-        <v>0.862</v>
+        <v>0.86199999999999999</v>
       </c>
       <c r="M22">
-        <v>0.956</v>
+        <v>0.95599999999999996</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -1680,16 +1630,16 @@
         <v>38270.1</v>
       </c>
       <c r="U22">
-        <v>128.932</v>
+        <v>128.93199999999999</v>
       </c>
       <c r="W22">
-        <v>0.162</v>
+        <v>0.16200000000000001</v>
       </c>
       <c r="X22">
-        <v>0.825</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>0.82499999999999996</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>1971</v>
       </c>
@@ -1703,13 +1653,13 @@
         <v>0.219</v>
       </c>
       <c r="F23">
-        <v>0.726</v>
+        <v>0.72599999999999998</v>
       </c>
       <c r="H23">
         <v>7124.4</v>
       </c>
       <c r="I23">
-        <v>126.353</v>
+        <v>126.35299999999999</v>
       </c>
       <c r="K23">
         <v>0.22</v>
@@ -1718,7 +1668,7 @@
         <v>0.746</v>
       </c>
       <c r="M23">
-        <v>0.854</v>
+        <v>0.85399999999999998</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -1733,10 +1683,10 @@
         <v>0.218</v>
       </c>
       <c r="X23">
-        <v>0.718</v>
-      </c>
-    </row>
-    <row r="24">
+        <v>0.71799999999999997</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>1972</v>
       </c>
@@ -1747,7 +1697,7 @@
         <v>118.413</v>
       </c>
       <c r="E24">
-        <v>0.237</v>
+        <v>0.23699999999999999</v>
       </c>
       <c r="F24">
         <v>0.62</v>
@@ -1762,10 +1712,10 @@
         <v>0.247</v>
       </c>
       <c r="L24">
-        <v>0.606</v>
+        <v>0.60599999999999998</v>
       </c>
       <c r="M24">
-        <v>0.864</v>
+        <v>0.86399999999999999</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -1777,13 +1727,13 @@
         <v>119.157</v>
       </c>
       <c r="W24">
-        <v>0.233</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="X24">
         <v>0.627</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>1973</v>
       </c>
@@ -1794,25 +1744,25 @@
         <v>101.858</v>
       </c>
       <c r="E25">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="F25">
-        <v>0.449</v>
+        <v>0.44900000000000001</v>
       </c>
       <c r="H25">
         <v>5732.8</v>
       </c>
       <c r="I25">
-        <v>121.698</v>
+        <v>121.69799999999999</v>
       </c>
       <c r="K25">
         <v>0.248</v>
       </c>
       <c r="L25">
-        <v>0.641</v>
+        <v>0.64100000000000001</v>
       </c>
       <c r="M25">
-        <v>0.895</v>
+        <v>0.89500000000000002</v>
       </c>
       <c r="N25">
         <v>0</v>
@@ -1821,16 +1771,16 @@
         <v>50929.2</v>
       </c>
       <c r="U25">
-        <v>98.07899999999999</v>
+        <v>98.078999999999994</v>
       </c>
       <c r="W25">
-        <v>0.237</v>
+        <v>0.23699999999999999</v>
       </c>
       <c r="X25">
-        <v>0.413</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>0.41299999999999998</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>1974</v>
       </c>
@@ -1838,28 +1788,28 @@
         <v>63702.9</v>
       </c>
       <c r="C26">
-        <v>97.54300000000001</v>
+        <v>97.543000000000006</v>
       </c>
       <c r="E26">
         <v>0.246</v>
       </c>
       <c r="F26">
-        <v>0.447</v>
+        <v>0.44700000000000001</v>
       </c>
       <c r="H26">
         <v>1878</v>
       </c>
       <c r="I26">
-        <v>120.195</v>
+        <v>120.19499999999999</v>
       </c>
       <c r="K26">
-        <v>0.208</v>
+        <v>0.20799999999999999</v>
       </c>
       <c r="L26">
-        <v>0.722</v>
+        <v>0.72199999999999998</v>
       </c>
       <c r="M26">
-        <v>0.834</v>
+        <v>0.83399999999999996</v>
       </c>
       <c r="N26">
         <v>0</v>
@@ -1868,16 +1818,16 @@
         <v>61824.9</v>
       </c>
       <c r="U26">
-        <v>93.767</v>
+        <v>93.766999999999996</v>
       </c>
       <c r="W26">
         <v>0.252</v>
       </c>
       <c r="X26">
-        <v>0.401</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>0.40100000000000002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>1975</v>
       </c>
@@ -1885,34 +1835,34 @@
         <v>60627.1</v>
       </c>
       <c r="C27">
-        <v>117.737</v>
+        <v>117.73699999999999</v>
       </c>
       <c r="E27">
         <v>0.185</v>
       </c>
       <c r="F27">
-        <v>0.659</v>
+        <v>0.65900000000000003</v>
       </c>
       <c r="H27">
         <v>6697.5</v>
       </c>
       <c r="I27">
-        <v>129.151</v>
+        <v>129.15100000000001</v>
       </c>
       <c r="K27">
-        <v>0.205</v>
+        <v>0.20499999999999999</v>
       </c>
       <c r="L27">
-        <v>0.806</v>
+        <v>0.80600000000000005</v>
       </c>
       <c r="M27">
-        <v>0.671</v>
+        <v>0.67100000000000004</v>
       </c>
       <c r="N27">
         <v>0</v>
       </c>
       <c r="T27">
-        <v>53929.6</v>
+        <v>53929.599999999999</v>
       </c>
       <c r="U27">
         <v>115.752</v>
@@ -1921,10 +1871,10 @@
         <v>0.182</v>
       </c>
       <c r="X27">
-        <v>0.634</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>0.63400000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>1976</v>
       </c>
@@ -1932,13 +1882,13 @@
         <v>44668.1</v>
       </c>
       <c r="C28">
-        <v>111.677</v>
+        <v>111.67700000000001</v>
       </c>
       <c r="E28">
         <v>0.184</v>
       </c>
       <c r="F28">
-        <v>0.607</v>
+        <v>0.60699999999999998</v>
       </c>
       <c r="H28">
         <v>1644</v>
@@ -1950,10 +1900,10 @@
         <v>0.187</v>
       </c>
       <c r="L28">
-        <v>0.826</v>
+        <v>0.82599999999999996</v>
       </c>
       <c r="M28">
-        <v>0.722</v>
+        <v>0.72199999999999998</v>
       </c>
       <c r="N28">
         <v>0</v>
@@ -1968,15 +1918,15 @@
         <v>0.183</v>
       </c>
       <c r="X28">
-        <v>0.572</v>
-      </c>
-    </row>
-    <row r="29">
+        <v>0.57199999999999995</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>1977</v>
       </c>
       <c r="B29">
-        <v>54735.2</v>
+        <v>54735.199999999997</v>
       </c>
       <c r="C29">
         <v>103.069</v>
@@ -1985,22 +1935,22 @@
         <v>0.2</v>
       </c>
       <c r="F29">
-        <v>0.528</v>
+        <v>0.52800000000000002</v>
       </c>
       <c r="H29">
         <v>4339</v>
       </c>
       <c r="I29">
-        <v>133.493</v>
+        <v>133.49299999999999</v>
       </c>
       <c r="K29">
         <v>0.161</v>
       </c>
       <c r="L29">
-        <v>0.868</v>
+        <v>0.86799999999999999</v>
       </c>
       <c r="M29">
-        <v>1.058</v>
+        <v>1.0580000000000001</v>
       </c>
       <c r="N29">
         <v>0</v>
@@ -2009,16 +1959,16 @@
         <v>50396.2</v>
       </c>
       <c r="U29">
-        <v>99.143</v>
+        <v>99.143000000000001</v>
       </c>
       <c r="W29">
-        <v>0.205</v>
+        <v>0.20499999999999999</v>
       </c>
       <c r="X29">
-        <v>0.484</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>0.48399999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>1978</v>
       </c>
@@ -2029,25 +1979,25 @@
         <v>113.932</v>
       </c>
       <c r="E30">
-        <v>0.205</v>
+        <v>0.20499999999999999</v>
       </c>
       <c r="F30">
-        <v>0.642</v>
+        <v>0.64200000000000002</v>
       </c>
       <c r="H30">
         <v>2875.2</v>
       </c>
       <c r="I30">
-        <v>128.234</v>
+        <v>128.23400000000001</v>
       </c>
       <c r="K30">
-        <v>0.168</v>
+        <v>0.16800000000000001</v>
       </c>
       <c r="L30">
-        <v>0.855</v>
+        <v>0.85499999999999998</v>
       </c>
       <c r="M30">
-        <v>0.885</v>
+        <v>0.88500000000000001</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -2056,16 +2006,16 @@
         <v>49556.3</v>
       </c>
       <c r="U30">
-        <v>111.207</v>
+        <v>111.20699999999999</v>
       </c>
       <c r="W30">
-        <v>0.212</v>
+        <v>0.21199999999999999</v>
       </c>
       <c r="X30">
-        <v>0.602</v>
-      </c>
-    </row>
-    <row r="31">
+        <v>0.60199999999999998</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>1979</v>
       </c>
@@ -2079,19 +2029,19 @@
         <v>0.221</v>
       </c>
       <c r="F31">
-        <v>0.464</v>
+        <v>0.46400000000000002</v>
       </c>
       <c r="H31">
-        <v>4241.6</v>
+        <v>4241.6000000000004</v>
       </c>
       <c r="I31">
-        <v>131.89</v>
+        <v>131.88999999999999</v>
       </c>
       <c r="K31">
-        <v>0.169</v>
+        <v>0.16900000000000001</v>
       </c>
       <c r="L31">
-        <v>0.854</v>
+        <v>0.85399999999999998</v>
       </c>
       <c r="M31">
         <v>1.587</v>
@@ -2100,19 +2050,19 @@
         <v>0</v>
       </c>
       <c r="T31">
-        <v>41588.4</v>
+        <v>41588.400000000001</v>
       </c>
       <c r="U31">
-        <v>97.833</v>
+        <v>97.832999999999998</v>
       </c>
       <c r="W31">
-        <v>0.228</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="X31">
-        <v>0.412</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>0.41199999999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>1980</v>
       </c>
@@ -2120,13 +2070,13 @@
         <v>63596.4</v>
       </c>
       <c r="C32">
-        <v>101.865</v>
+        <v>101.86499999999999</v>
       </c>
       <c r="E32">
-        <v>0.259</v>
+        <v>0.25900000000000001</v>
       </c>
       <c r="F32">
-        <v>0.529</v>
+        <v>0.52900000000000003</v>
       </c>
       <c r="H32">
         <v>10331</v>
@@ -2135,10 +2085,10 @@
         <v>133.631</v>
       </c>
       <c r="K32">
-        <v>0.164</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="L32">
-        <v>0.957</v>
+        <v>0.95699999999999996</v>
       </c>
       <c r="M32">
         <v>1.526</v>
@@ -2150,16 +2100,16 @@
         <v>53265.4</v>
       </c>
       <c r="U32">
-        <v>96.34099999999999</v>
+        <v>96.340999999999994</v>
       </c>
       <c r="W32">
-        <v>0.276</v>
+        <v>0.27600000000000002</v>
       </c>
       <c r="X32">
-        <v>0.455</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>0.45500000000000002</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>1981</v>
       </c>
@@ -2167,28 +2117,28 @@
         <v>67772.7</v>
       </c>
       <c r="C33">
-        <v>107.594</v>
+        <v>107.59399999999999</v>
       </c>
       <c r="E33">
         <v>0.23</v>
       </c>
       <c r="F33">
-        <v>0.546</v>
+        <v>0.54600000000000004</v>
       </c>
       <c r="H33">
-        <v>9622.700000000001</v>
+        <v>9622.7000000000007</v>
       </c>
       <c r="I33">
         <v>124.471</v>
       </c>
       <c r="K33">
-        <v>0.175</v>
+        <v>0.17499999999999999</v>
       </c>
       <c r="L33">
-        <v>0.8090000000000001</v>
+        <v>0.80900000000000005</v>
       </c>
       <c r="M33">
-        <v>1.281</v>
+        <v>1.2809999999999999</v>
       </c>
       <c r="N33">
         <v>0</v>
@@ -2200,18 +2150,18 @@
         <v>105.417</v>
       </c>
       <c r="W33">
-        <v>0.237</v>
+        <v>0.23699999999999999</v>
       </c>
       <c r="X33">
-        <v>0.513</v>
-      </c>
-    </row>
-    <row r="34">
+        <v>0.51300000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>1982</v>
       </c>
       <c r="B34">
-        <v>73556.89999999999</v>
+        <v>73556.899999999994</v>
       </c>
       <c r="C34">
         <v>105.59</v>
@@ -2220,7 +2170,7 @@
         <v>0.245</v>
       </c>
       <c r="F34">
-        <v>0.512</v>
+        <v>0.51200000000000001</v>
       </c>
       <c r="H34">
         <v>24527.1</v>
@@ -2232,7 +2182,7 @@
         <v>0.191</v>
       </c>
       <c r="L34">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="M34">
         <v>1.302</v>
@@ -2253,12 +2203,12 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>1983</v>
       </c>
       <c r="B35">
-        <v>59434.4</v>
+        <v>59434.400000000001</v>
       </c>
       <c r="C35">
         <v>104.884</v>
@@ -2270,7 +2220,7 @@
         <v>0.54</v>
       </c>
       <c r="H35">
-        <v>9511.799999999999</v>
+        <v>9511.7999999999993</v>
       </c>
       <c r="I35">
         <v>127.49</v>
@@ -2279,10 +2229,10 @@
         <v>0.186</v>
       </c>
       <c r="L35">
-        <v>0.827</v>
+        <v>0.82699999999999996</v>
       </c>
       <c r="M35">
-        <v>1.271</v>
+        <v>1.2709999999999999</v>
       </c>
       <c r="N35">
         <v>0</v>
@@ -2300,7 +2250,7 @@
         <v>0.502</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>1984</v>
       </c>
@@ -2311,25 +2261,25 @@
         <v>111.316</v>
       </c>
       <c r="E36">
-        <v>0.211</v>
+        <v>0.21099999999999999</v>
       </c>
       <c r="F36">
         <v>0.621</v>
       </c>
       <c r="H36">
-        <v>16972.4</v>
+        <v>16972.400000000001</v>
       </c>
       <c r="I36">
         <v>126.857</v>
       </c>
       <c r="K36">
-        <v>0.176</v>
+        <v>0.17599999999999999</v>
       </c>
       <c r="L36">
-        <v>0.799</v>
+        <v>0.79900000000000004</v>
       </c>
       <c r="M36">
-        <v>1.495</v>
+        <v>1.4950000000000001</v>
       </c>
       <c r="N36">
         <v>0</v>
@@ -2338,30 +2288,30 @@
         <v>54005.1</v>
       </c>
       <c r="U36">
-        <v>109.311</v>
+        <v>109.31100000000001</v>
       </c>
       <c r="W36">
         <v>0.215</v>
       </c>
       <c r="X36">
-        <v>0.598</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>0.59799999999999998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>1985</v>
       </c>
       <c r="B37">
-        <v>78009.10000000001</v>
+        <v>78009.100000000006</v>
       </c>
       <c r="C37">
         <v>100.765</v>
       </c>
       <c r="E37">
-        <v>0.207</v>
+        <v>0.20699999999999999</v>
       </c>
       <c r="F37">
-        <v>0.475</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="H37">
         <v>24878.6</v>
@@ -2370,13 +2320,13 @@
         <v>123.378</v>
       </c>
       <c r="K37">
-        <v>0.177</v>
+        <v>0.17699999999999999</v>
       </c>
       <c r="L37">
-        <v>0.776</v>
+        <v>0.77600000000000002</v>
       </c>
       <c r="M37">
-        <v>1.576</v>
+        <v>1.5760000000000001</v>
       </c>
       <c r="N37">
         <v>0</v>
@@ -2385,7 +2335,7 @@
         <v>53130.5</v>
       </c>
       <c r="U37">
-        <v>98.31999999999999</v>
+        <v>98.32</v>
       </c>
       <c r="W37">
         <v>0.21</v>
@@ -2394,7 +2344,7 @@
         <v>0.442</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>1986</v>
       </c>
@@ -2408,22 +2358,22 @@
         <v>0.222</v>
       </c>
       <c r="F38">
-        <v>0.5580000000000001</v>
+        <v>0.55800000000000005</v>
       </c>
       <c r="H38">
         <v>15716.4</v>
       </c>
       <c r="I38">
-        <v>126.835</v>
+        <v>126.83499999999999</v>
       </c>
       <c r="K38">
         <v>0.188</v>
       </c>
       <c r="L38">
-        <v>0.8120000000000001</v>
+        <v>0.81200000000000006</v>
       </c>
       <c r="M38">
-        <v>1.485</v>
+        <v>1.4850000000000001</v>
       </c>
       <c r="N38">
         <v>0</v>
@@ -2432,16 +2382,16 @@
         <v>49716.2</v>
       </c>
       <c r="U38">
-        <v>102.043</v>
+        <v>102.04300000000001</v>
       </c>
       <c r="W38">
-        <v>0.226</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="X38">
-        <v>0.526</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>0.52600000000000002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>1987</v>
       </c>
@@ -2449,7 +2399,7 @@
         <v>57322.5</v>
       </c>
       <c r="C39">
-        <v>103.106</v>
+        <v>103.10599999999999</v>
       </c>
       <c r="E39">
         <v>0.217</v>
@@ -2467,7 +2417,7 @@
         <v>0.182</v>
       </c>
       <c r="L39">
-        <v>0.777</v>
+        <v>0.77700000000000002</v>
       </c>
       <c r="M39">
         <v>1.871</v>
@@ -2479,30 +2429,30 @@
         <v>44862.2</v>
       </c>
       <c r="U39">
-        <v>100.391</v>
+        <v>100.39100000000001</v>
       </c>
       <c r="W39">
         <v>0.221</v>
       </c>
       <c r="X39">
-        <v>0.469</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>0.46899999999999997</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>1988</v>
       </c>
       <c r="B40">
-        <v>66374.60000000001</v>
+        <v>66374.600000000006</v>
       </c>
       <c r="C40">
-        <v>96.946</v>
+        <v>96.945999999999998</v>
       </c>
       <c r="E40">
-        <v>0.229</v>
+        <v>0.22900000000000001</v>
       </c>
       <c r="F40">
-        <v>0.447</v>
+        <v>0.44700000000000001</v>
       </c>
       <c r="H40">
         <v>24028.3</v>
@@ -2511,13 +2461,13 @@
         <v>123.824</v>
       </c>
       <c r="K40">
-        <v>0.169</v>
+        <v>0.16900000000000001</v>
       </c>
       <c r="L40">
-        <v>0.785</v>
+        <v>0.78500000000000003</v>
       </c>
       <c r="M40">
-        <v>1.759</v>
+        <v>1.7589999999999999</v>
       </c>
       <c r="N40">
         <v>0</v>
@@ -2526,36 +2476,36 @@
         <v>42346.3</v>
       </c>
       <c r="U40">
-        <v>93.95999999999999</v>
+        <v>93.96</v>
       </c>
       <c r="W40">
-        <v>0.236</v>
+        <v>0.23599999999999999</v>
       </c>
       <c r="X40">
-        <v>0.409</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>0.40899999999999997</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>1989</v>
       </c>
       <c r="B41">
-        <v>78721.39999999999</v>
+        <v>78721.399999999994</v>
       </c>
       <c r="C41">
-        <v>102.061</v>
+        <v>102.06100000000001</v>
       </c>
       <c r="E41">
-        <v>0.204</v>
+        <v>0.20399999999999999</v>
       </c>
       <c r="F41">
-        <v>0.511</v>
+        <v>0.51100000000000001</v>
       </c>
       <c r="H41">
         <v>31661.9</v>
       </c>
       <c r="I41">
-        <v>128.743</v>
+        <v>128.74299999999999</v>
       </c>
       <c r="K41">
         <v>0.157</v>
@@ -2573,16 +2523,16 @@
         <v>47059.5</v>
       </c>
       <c r="U41">
-        <v>98.61799999999999</v>
+        <v>98.617999999999995</v>
       </c>
       <c r="W41">
         <v>0.21</v>
       </c>
       <c r="X41">
-        <v>0.463</v>
-      </c>
-    </row>
-    <row r="42">
+        <v>0.46300000000000002</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>1990</v>
       </c>
@@ -2593,10 +2543,10 @@
         <v>109.253</v>
       </c>
       <c r="E42">
-        <v>0.205</v>
+        <v>0.20499999999999999</v>
       </c>
       <c r="F42">
-        <v>0.5679999999999999</v>
+        <v>0.56799999999999995</v>
       </c>
       <c r="H42">
         <v>26431.1</v>
@@ -2605,10 +2555,10 @@
         <v>124.92</v>
       </c>
       <c r="K42">
-        <v>0.171</v>
+        <v>0.17100000000000001</v>
       </c>
       <c r="L42">
-        <v>0.783</v>
+        <v>0.78300000000000003</v>
       </c>
       <c r="M42">
         <v>1.2</v>
@@ -2620,42 +2570,42 @@
         <v>58832.6</v>
       </c>
       <c r="U42">
-        <v>106.528</v>
+        <v>106.52800000000001</v>
       </c>
       <c r="W42">
-        <v>0.211</v>
+        <v>0.21099999999999999</v>
       </c>
       <c r="X42">
         <v>0.53</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>1991</v>
       </c>
       <c r="B43">
-        <v>97211.2</v>
+        <v>97211.199999999997</v>
       </c>
       <c r="C43">
         <v>93.378</v>
       </c>
       <c r="E43">
-        <v>0.211</v>
+        <v>0.21099999999999999</v>
       </c>
       <c r="F43">
-        <v>0.426</v>
+        <v>0.42599999999999999</v>
       </c>
       <c r="H43">
         <v>21041.9</v>
       </c>
       <c r="I43">
-        <v>128.378</v>
+        <v>128.37799999999999</v>
       </c>
       <c r="K43">
         <v>0.152</v>
       </c>
       <c r="L43">
-        <v>0.864</v>
+        <v>0.86399999999999999</v>
       </c>
       <c r="M43">
         <v>1.22</v>
@@ -2664,28 +2614,28 @@
         <v>14048.6</v>
       </c>
       <c r="O43">
-        <v>55.229</v>
+        <v>55.228999999999999</v>
       </c>
       <c r="Q43">
-        <v>0.333</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="R43">
-        <v>0.028</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="T43">
         <v>62120.7</v>
       </c>
       <c r="U43">
-        <v>93.828</v>
+        <v>93.828000000000003</v>
       </c>
       <c r="W43">
-        <v>0.202</v>
+        <v>0.20200000000000001</v>
       </c>
       <c r="X43">
-        <v>0.421</v>
-      </c>
-    </row>
-    <row r="44">
+        <v>0.42099999999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>1992</v>
       </c>
@@ -2693,13 +2643,13 @@
         <v>100106</v>
       </c>
       <c r="C44">
-        <v>96.658</v>
+        <v>96.658000000000001</v>
       </c>
       <c r="E44">
         <v>0.216</v>
       </c>
       <c r="F44">
-        <v>0.429</v>
+        <v>0.42899999999999999</v>
       </c>
       <c r="H44">
         <v>24247.3</v>
@@ -2708,40 +2658,40 @@
         <v>127.595</v>
       </c>
       <c r="K44">
-        <v>0.169</v>
+        <v>0.16900000000000001</v>
       </c>
       <c r="L44">
-        <v>0.824</v>
+        <v>0.82399999999999995</v>
       </c>
       <c r="M44">
-        <v>1.078</v>
+        <v>1.0780000000000001</v>
       </c>
       <c r="N44">
         <v>16239.7</v>
       </c>
       <c r="O44">
-        <v>56.056</v>
+        <v>56.055999999999997</v>
       </c>
       <c r="Q44">
-        <v>0.353</v>
+        <v>0.35299999999999998</v>
       </c>
       <c r="R44">
-        <v>0.042</v>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="T44">
         <v>59619</v>
       </c>
       <c r="U44">
-        <v>97.867</v>
+        <v>97.867000000000004</v>
       </c>
       <c r="W44">
-        <v>0.205</v>
+        <v>0.20499999999999999</v>
       </c>
       <c r="X44">
-        <v>0.428</v>
-      </c>
-    </row>
-    <row r="45">
+        <v>0.42799999999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>1993</v>
       </c>
@@ -2749,16 +2699,16 @@
         <v>113789.7</v>
       </c>
       <c r="C45">
-        <v>95.38200000000001</v>
+        <v>95.382000000000005</v>
       </c>
       <c r="E45">
-        <v>0.229</v>
+        <v>0.22900000000000001</v>
       </c>
       <c r="F45">
         <v>0.435</v>
       </c>
       <c r="H45">
-        <v>25717.2</v>
+        <v>25717.200000000001</v>
       </c>
       <c r="I45">
         <v>127.61</v>
@@ -2767,22 +2717,22 @@
         <v>0.19</v>
       </c>
       <c r="L45">
-        <v>0.8129999999999999</v>
+        <v>0.81299999999999994</v>
       </c>
       <c r="M45">
         <v>1.2</v>
       </c>
       <c r="N45">
-        <v>24272.4</v>
+        <v>24272.400000000001</v>
       </c>
       <c r="O45">
-        <v>56.815</v>
+        <v>56.814999999999998</v>
       </c>
       <c r="Q45">
-        <v>0.354</v>
+        <v>0.35399999999999998</v>
       </c>
       <c r="R45">
-        <v>0.034</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="T45">
         <v>63800.1</v>
@@ -2797,7 +2747,7 @@
         <v>0.438</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>1994</v>
       </c>
@@ -2805,22 +2755,22 @@
         <v>134932.1</v>
       </c>
       <c r="C46">
-        <v>92.407</v>
+        <v>92.406999999999996</v>
       </c>
       <c r="E46">
-        <v>0.211</v>
+        <v>0.21099999999999999</v>
       </c>
       <c r="F46">
         <v>0.378</v>
       </c>
       <c r="H46">
-        <v>27781.2</v>
+        <v>27781.200000000001</v>
       </c>
       <c r="I46">
-        <v>132.681</v>
+        <v>132.68100000000001</v>
       </c>
       <c r="K46">
-        <v>0.164</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="L46">
         <v>0.878</v>
@@ -2832,28 +2782,28 @@
         <v>28389.7</v>
       </c>
       <c r="O46">
-        <v>56.288</v>
+        <v>56.287999999999997</v>
       </c>
       <c r="Q46">
         <v>0.375</v>
       </c>
       <c r="R46">
-        <v>0.036</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="T46">
         <v>78761.2</v>
       </c>
       <c r="U46">
-        <v>91.904</v>
+        <v>91.903999999999996</v>
       </c>
       <c r="W46">
-        <v>0.197</v>
+        <v>0.19700000000000001</v>
       </c>
       <c r="X46">
-        <v>0.359</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>0.35899999999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>1995</v>
       </c>
@@ -2861,40 +2811,40 @@
         <v>128046.9</v>
       </c>
       <c r="C47">
-        <v>95.77800000000001</v>
+        <v>95.778000000000006</v>
       </c>
       <c r="E47">
-        <v>0.227</v>
+        <v>0.22700000000000001</v>
       </c>
       <c r="F47">
-        <v>0.414</v>
+        <v>0.41399999999999998</v>
       </c>
       <c r="H47">
         <v>26995</v>
       </c>
       <c r="I47">
-        <v>136.117</v>
+        <v>136.11699999999999</v>
       </c>
       <c r="K47">
         <v>0.184</v>
       </c>
       <c r="L47">
-        <v>0.864</v>
+        <v>0.86399999999999999</v>
       </c>
       <c r="M47">
-        <v>1.241</v>
+        <v>1.2410000000000001</v>
       </c>
       <c r="N47">
         <v>23113.4</v>
       </c>
       <c r="O47">
-        <v>57.133</v>
+        <v>57.133000000000003</v>
       </c>
       <c r="Q47">
-        <v>0.363</v>
+        <v>0.36299999999999999</v>
       </c>
       <c r="R47">
-        <v>0.041</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="T47">
         <v>77938.5</v>
@@ -2906,10 +2856,10 @@
         <v>0.217</v>
       </c>
       <c r="X47">
-        <v>0.405</v>
-      </c>
-    </row>
-    <row r="48">
+        <v>0.40500000000000003</v>
+      </c>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>1996</v>
       </c>
@@ -2935,37 +2885,37 @@
         <v>0.17</v>
       </c>
       <c r="L48">
-        <v>0.911</v>
+        <v>0.91100000000000003</v>
       </c>
       <c r="M48">
-        <v>0.864</v>
+        <v>0.86399999999999999</v>
       </c>
       <c r="N48">
         <v>22402.2</v>
       </c>
       <c r="O48">
-        <v>57.556</v>
+        <v>57.555999999999997</v>
       </c>
       <c r="Q48">
-        <v>0.359</v>
+        <v>0.35899999999999999</v>
       </c>
       <c r="R48">
-        <v>0.046</v>
+        <v>4.5999999999999999E-2</v>
       </c>
       <c r="T48">
-        <v>72945.89999999999</v>
+        <v>72945.899999999994</v>
       </c>
       <c r="U48">
         <v>102.292</v>
       </c>
       <c r="W48">
-        <v>0.202</v>
+        <v>0.20200000000000001</v>
       </c>
       <c r="X48">
         <v>0.52</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>1997</v>
       </c>
@@ -2973,13 +2923,13 @@
         <v>110254.3</v>
       </c>
       <c r="C49">
-        <v>86.947</v>
+        <v>86.947000000000003</v>
       </c>
       <c r="E49">
         <v>0.252</v>
       </c>
       <c r="F49">
-        <v>0.341</v>
+        <v>0.34100000000000003</v>
       </c>
       <c r="H49">
         <v>18052.8</v>
@@ -2991,37 +2941,37 @@
         <v>0.157</v>
       </c>
       <c r="L49">
-        <v>0.912</v>
+        <v>0.91200000000000003</v>
       </c>
       <c r="M49">
-        <v>0.773</v>
+        <v>0.77300000000000002</v>
       </c>
       <c r="N49">
         <v>14110.8</v>
       </c>
       <c r="O49">
-        <v>53.468</v>
+        <v>53.468000000000004</v>
       </c>
       <c r="Q49">
         <v>0.378</v>
       </c>
       <c r="R49">
-        <v>0.034</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="T49">
         <v>78090.7</v>
       </c>
       <c r="U49">
-        <v>85.041</v>
+        <v>85.040999999999997</v>
       </c>
       <c r="W49">
         <v>0.248</v>
       </c>
       <c r="X49">
-        <v>0.299</v>
-      </c>
-    </row>
-    <row r="50">
+        <v>0.29899999999999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>1998</v>
       </c>
@@ -3029,55 +2979,55 @@
         <v>107952.4</v>
       </c>
       <c r="C50">
-        <v>87.92700000000001</v>
+        <v>87.927000000000007</v>
       </c>
       <c r="E50">
         <v>0.216</v>
       </c>
       <c r="F50">
-        <v>0.333</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="H50">
         <v>16131.2</v>
       </c>
       <c r="I50">
-        <v>129.141</v>
+        <v>129.14099999999999</v>
       </c>
       <c r="K50">
-        <v>0.179</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="L50">
-        <v>0.819</v>
+        <v>0.81899999999999995</v>
       </c>
       <c r="M50">
-        <v>0.803</v>
+        <v>0.80300000000000005</v>
       </c>
       <c r="N50">
         <v>10731.1</v>
       </c>
       <c r="O50">
-        <v>48.399</v>
+        <v>48.399000000000001</v>
       </c>
       <c r="Q50">
-        <v>0.239</v>
+        <v>0.23899999999999999</v>
       </c>
       <c r="R50">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="T50">
-        <v>81090.10000000001</v>
+        <v>81090.100000000006</v>
       </c>
       <c r="U50">
-        <v>87.633</v>
+        <v>87.632999999999996</v>
       </c>
       <c r="W50">
         <v>0.218</v>
       </c>
       <c r="X50">
-        <v>0.306</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>0.30599999999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>1999</v>
       </c>
@@ -3088,25 +3038,25 @@
         <v>101.131</v>
       </c>
       <c r="E51">
-        <v>0.204</v>
+        <v>0.20399999999999999</v>
       </c>
       <c r="F51">
-        <v>0.491</v>
+        <v>0.49099999999999999</v>
       </c>
       <c r="H51">
         <v>14764.9</v>
       </c>
       <c r="I51">
-        <v>126.085</v>
+        <v>126.08499999999999</v>
       </c>
       <c r="K51">
         <v>0.158</v>
       </c>
       <c r="L51">
-        <v>0.852</v>
+        <v>0.85199999999999998</v>
       </c>
       <c r="M51">
-        <v>0.793</v>
+        <v>0.79300000000000004</v>
       </c>
       <c r="N51">
         <v>12027.7</v>
@@ -3118,7 +3068,7 @@
         <v>0.312</v>
       </c>
       <c r="R51">
-        <v>0.022</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="T51">
         <v>94631.8</v>
@@ -3127,13 +3077,13 @@
         <v>104.35</v>
       </c>
       <c r="W51">
-        <v>0.195</v>
+        <v>0.19500000000000001</v>
       </c>
       <c r="X51">
-        <v>0.507</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>0.50700000000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>2000</v>
       </c>
@@ -3141,55 +3091,55 @@
         <v>103433.7</v>
       </c>
       <c r="C52">
-        <v>94.629</v>
+        <v>94.629000000000005</v>
       </c>
       <c r="E52">
-        <v>0.232</v>
+        <v>0.23200000000000001</v>
       </c>
       <c r="F52">
-        <v>0.424</v>
+        <v>0.42399999999999999</v>
       </c>
       <c r="H52">
         <v>17231.3</v>
       </c>
       <c r="I52">
-        <v>128.778</v>
+        <v>128.77799999999999</v>
       </c>
       <c r="K52">
         <v>0.158</v>
       </c>
       <c r="L52">
-        <v>0.862</v>
+        <v>0.86199999999999999</v>
       </c>
       <c r="M52">
-        <v>0.803</v>
+        <v>0.80300000000000005</v>
       </c>
       <c r="N52">
         <v>12390.4</v>
       </c>
       <c r="O52">
-        <v>50.477</v>
+        <v>50.476999999999997</v>
       </c>
       <c r="Q52">
         <v>0.249</v>
       </c>
       <c r="R52">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="T52">
         <v>73812</v>
       </c>
       <c r="U52">
-        <v>96.297</v>
+        <v>96.296999999999997</v>
       </c>
       <c r="W52">
-        <v>0.242</v>
+        <v>0.24199999999999999</v>
       </c>
       <c r="X52">
         <v>0.42</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>2001</v>
       </c>
@@ -3200,10 +3150,10 @@
         <v>96.28</v>
       </c>
       <c r="E53">
-        <v>0.232</v>
+        <v>0.23200000000000001</v>
       </c>
       <c r="F53">
-        <v>0.454</v>
+        <v>0.45400000000000001</v>
       </c>
       <c r="H53">
         <v>11798.1</v>
@@ -3215,48 +3165,48 @@
         <v>0.16</v>
       </c>
       <c r="L53">
-        <v>0.826</v>
+        <v>0.82599999999999996</v>
       </c>
       <c r="M53">
-        <v>0.671</v>
+        <v>0.67100000000000004</v>
       </c>
       <c r="N53">
         <v>11308.5</v>
       </c>
       <c r="O53">
-        <v>52.536</v>
+        <v>52.536000000000001</v>
       </c>
       <c r="Q53">
         <v>0.311</v>
       </c>
       <c r="R53">
-        <v>0.018</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="T53">
-        <v>68529.10000000001</v>
+        <v>68529.100000000006</v>
       </c>
       <c r="U53">
-        <v>98.057</v>
+        <v>98.057000000000002</v>
       </c>
       <c r="W53">
-        <v>0.231</v>
+        <v>0.23100000000000001</v>
       </c>
       <c r="X53">
-        <v>0.462</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>0.46200000000000002</v>
+      </c>
+    </row>
+    <row r="54" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>2002</v>
       </c>
       <c r="B54">
-        <v>75801.60000000001</v>
+        <v>75801.600000000006</v>
       </c>
       <c r="C54">
-        <v>99.574</v>
+        <v>99.573999999999998</v>
       </c>
       <c r="E54">
-        <v>0.213</v>
+        <v>0.21299999999999999</v>
       </c>
       <c r="F54">
         <v>0.497</v>
@@ -3265,43 +3215,43 @@
         <v>9906.4</v>
       </c>
       <c r="I54">
-        <v>131.08</v>
+        <v>131.08000000000001</v>
       </c>
       <c r="K54">
-        <v>0.162</v>
+        <v>0.16200000000000001</v>
       </c>
       <c r="L54">
         <v>0.873</v>
       </c>
       <c r="M54">
-        <v>0.712</v>
+        <v>0.71199999999999997</v>
       </c>
       <c r="N54">
         <v>10018.9</v>
       </c>
       <c r="O54">
-        <v>50.891</v>
+        <v>50.890999999999998</v>
       </c>
       <c r="Q54">
-        <v>0.262</v>
+        <v>0.26200000000000001</v>
       </c>
       <c r="R54">
-        <v>0.008999999999999999</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="T54">
         <v>55876.3</v>
       </c>
       <c r="U54">
-        <v>102.028</v>
+        <v>102.02800000000001</v>
       </c>
       <c r="W54">
-        <v>0.213</v>
+        <v>0.21299999999999999</v>
       </c>
       <c r="X54">
-        <v>0.513</v>
-      </c>
-    </row>
-    <row r="55">
+        <v>0.51300000000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>2003</v>
       </c>
@@ -3315,7 +3265,7 @@
         <v>0.21</v>
       </c>
       <c r="F55">
-        <v>0.467</v>
+        <v>0.46700000000000003</v>
       </c>
       <c r="H55">
         <v>11797</v>
@@ -3324,13 +3274,13 @@
         <v>136.286</v>
       </c>
       <c r="K55">
-        <v>0.169</v>
+        <v>0.16900000000000001</v>
       </c>
       <c r="L55">
-        <v>0.902</v>
+        <v>0.90200000000000002</v>
       </c>
       <c r="M55">
-        <v>0.732</v>
+        <v>0.73199999999999998</v>
       </c>
       <c r="N55">
         <v>11107.9</v>
@@ -3339,39 +3289,39 @@
         <v>49.186</v>
       </c>
       <c r="Q55">
-        <v>0.261</v>
+        <v>0.26100000000000001</v>
       </c>
       <c r="R55">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="T55">
         <v>64690.1</v>
       </c>
       <c r="U55">
-        <v>97.483</v>
+        <v>97.483000000000004</v>
       </c>
       <c r="W55">
-        <v>0.208</v>
+        <v>0.20799999999999999</v>
       </c>
       <c r="X55">
         <v>0.47</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>2004</v>
       </c>
       <c r="B56">
-        <v>90042.89999999999</v>
+        <v>90042.9</v>
       </c>
       <c r="C56">
-        <v>97.68300000000001</v>
+        <v>97.683000000000007</v>
       </c>
       <c r="E56">
-        <v>0.227</v>
+        <v>0.22700000000000001</v>
       </c>
       <c r="F56">
-        <v>0.448</v>
+        <v>0.44800000000000001</v>
       </c>
       <c r="H56">
         <v>11466.1</v>
@@ -3380,10 +3330,10 @@
         <v>136.404</v>
       </c>
       <c r="K56">
-        <v>0.165</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="L56">
-        <v>0.898</v>
+        <v>0.89800000000000002</v>
       </c>
       <c r="M56">
         <v>0.59</v>
@@ -3392,33 +3342,33 @@
         <v>11338.2</v>
       </c>
       <c r="O56">
-        <v>50.461</v>
+        <v>50.460999999999999</v>
       </c>
       <c r="Q56">
-        <v>0.265</v>
+        <v>0.26500000000000001</v>
       </c>
       <c r="R56">
-        <v>0.008999999999999999</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="T56">
-        <v>67238.60000000001</v>
+        <v>67238.600000000006</v>
       </c>
       <c r="U56">
-        <v>98.746</v>
+        <v>98.745999999999995</v>
       </c>
       <c r="W56">
-        <v>0.231</v>
+        <v>0.23100000000000001</v>
       </c>
       <c r="X56">
-        <v>0.447</v>
-      </c>
-    </row>
-    <row r="57">
+        <v>0.44700000000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>2005</v>
       </c>
       <c r="B57">
-        <v>67953.39999999999</v>
+        <v>67953.399999999994</v>
       </c>
       <c r="C57">
         <v>101.873</v>
@@ -3427,34 +3377,34 @@
         <v>0.22</v>
       </c>
       <c r="F57">
-        <v>0.489</v>
+        <v>0.48899999999999999</v>
       </c>
       <c r="H57">
-        <v>8782.200000000001</v>
+        <v>8782.2000000000007</v>
       </c>
       <c r="I57">
         <v>138.834</v>
       </c>
       <c r="K57">
-        <v>0.163</v>
+        <v>0.16300000000000001</v>
       </c>
       <c r="L57">
-        <v>0.923</v>
+        <v>0.92300000000000004</v>
       </c>
       <c r="M57">
-        <v>0.681</v>
+        <v>0.68100000000000005</v>
       </c>
       <c r="N57">
-        <v>8601.700000000001</v>
+        <v>8601.7000000000007</v>
       </c>
       <c r="O57">
         <v>48.125</v>
       </c>
       <c r="Q57">
-        <v>0.236</v>
+        <v>0.23599999999999999</v>
       </c>
       <c r="R57">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="T57">
         <v>50569.5</v>
@@ -3466,10 +3416,10 @@
         <v>0.224</v>
       </c>
       <c r="X57">
-        <v>0.514</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>0.51400000000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>2006</v>
       </c>
@@ -3480,7 +3430,7 @@
         <v>103.661</v>
       </c>
       <c r="E58">
-        <v>0.205</v>
+        <v>0.20499999999999999</v>
       </c>
       <c r="F58">
         <v>0.499</v>
@@ -3495,10 +3445,10 @@
         <v>0.191</v>
       </c>
       <c r="L58">
-        <v>0.784</v>
+        <v>0.78400000000000003</v>
       </c>
       <c r="M58">
-        <v>0.763</v>
+        <v>0.76300000000000001</v>
       </c>
       <c r="N58">
         <v>7054.2</v>
@@ -3510,22 +3460,22 @@
         <v>0.251</v>
       </c>
       <c r="R58">
-        <v>0.008999999999999999</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="T58">
         <v>42927.1</v>
       </c>
       <c r="U58">
-        <v>107.743</v>
+        <v>107.74299999999999</v>
       </c>
       <c r="W58">
-        <v>0.201</v>
+        <v>0.20100000000000001</v>
       </c>
       <c r="X58">
-        <v>0.528</v>
-      </c>
-    </row>
-    <row r="59">
+        <v>0.52800000000000002</v>
+      </c>
+    </row>
+    <row r="59" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>2007</v>
       </c>
@@ -3539,34 +3489,34 @@
         <v>0.215</v>
       </c>
       <c r="F59">
-        <v>0.5679999999999999</v>
+        <v>0.56799999999999995</v>
       </c>
       <c r="H59">
         <v>12802.5</v>
       </c>
       <c r="I59">
-        <v>135.701</v>
+        <v>135.70099999999999</v>
       </c>
       <c r="K59">
         <v>0.159</v>
       </c>
       <c r="L59">
-        <v>0.893</v>
+        <v>0.89300000000000002</v>
       </c>
       <c r="M59">
-        <v>0.773</v>
+        <v>0.77300000000000002</v>
       </c>
       <c r="N59">
         <v>7777.3</v>
       </c>
       <c r="O59">
-        <v>48.337</v>
+        <v>48.337000000000003</v>
       </c>
       <c r="Q59">
-        <v>0.235</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="R59">
-        <v>0.005</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="T59">
         <v>49314.7</v>
@@ -3578,10 +3528,10 @@
         <v>0.219</v>
       </c>
       <c r="X59">
-        <v>0.577</v>
-      </c>
-    </row>
-    <row r="60">
+        <v>0.57699999999999996</v>
+      </c>
+    </row>
+    <row r="60" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>2008</v>
       </c>
@@ -3589,40 +3539,40 @@
         <v>63171.6</v>
       </c>
       <c r="C60">
-        <v>118.472</v>
+        <v>118.47199999999999</v>
       </c>
       <c r="E60">
-        <v>0.179</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="F60">
-        <v>0.6929999999999999</v>
+        <v>0.69299999999999995</v>
       </c>
       <c r="H60">
         <v>12220</v>
       </c>
       <c r="I60">
-        <v>136.301</v>
+        <v>136.30099999999999</v>
       </c>
       <c r="K60">
-        <v>0.181</v>
+        <v>0.18099999999999999</v>
       </c>
       <c r="L60">
         <v>0.87</v>
       </c>
       <c r="M60">
-        <v>0.651</v>
+        <v>0.65100000000000002</v>
       </c>
       <c r="N60">
         <v>10049.5</v>
       </c>
       <c r="O60">
-        <v>44.825</v>
+        <v>44.825000000000003</v>
       </c>
       <c r="Q60">
-        <v>0.231</v>
+        <v>0.23100000000000001</v>
       </c>
       <c r="R60">
-        <v>0.004</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="T60">
         <v>40902.1</v>
@@ -3631,13 +3581,13 @@
         <v>118.536</v>
       </c>
       <c r="W60">
-        <v>0.177</v>
+        <v>0.17699999999999999</v>
       </c>
       <c r="X60">
-        <v>0.6929999999999999</v>
-      </c>
-    </row>
-    <row r="61">
+        <v>0.69299999999999995</v>
+      </c>
+    </row>
+    <row r="61" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>2009</v>
       </c>
@@ -3648,22 +3598,22 @@
         <v>112.042</v>
       </c>
       <c r="E61">
-        <v>0.204</v>
+        <v>0.20399999999999999</v>
       </c>
       <c r="F61">
-        <v>0.587</v>
+        <v>0.58699999999999997</v>
       </c>
       <c r="H61">
         <v>13250.9</v>
       </c>
       <c r="I61">
-        <v>130.013</v>
+        <v>130.01300000000001</v>
       </c>
       <c r="K61">
-        <v>0.194</v>
+        <v>0.19400000000000001</v>
       </c>
       <c r="L61">
-        <v>0.783</v>
+        <v>0.78300000000000003</v>
       </c>
       <c r="M61">
         <v>0.59</v>
@@ -3672,13 +3622,13 @@
         <v>13171</v>
       </c>
       <c r="O61">
-        <v>49.077</v>
+        <v>49.076999999999998</v>
       </c>
       <c r="Q61">
-        <v>0.272</v>
+        <v>0.27200000000000002</v>
       </c>
       <c r="R61">
-        <v>0.013</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="T61">
         <v>50005.4</v>
@@ -3687,13 +3637,13 @@
         <v>116.327</v>
       </c>
       <c r="W61">
-        <v>0.199</v>
+        <v>0.19900000000000001</v>
       </c>
       <c r="X61">
         <v>0.623</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>2010</v>
       </c>
@@ -3707,19 +3657,19 @@
         <v>0.214</v>
       </c>
       <c r="F62">
-        <v>0.589</v>
+        <v>0.58899999999999997</v>
       </c>
       <c r="H62">
-        <v>10234.2</v>
+        <v>10234.200000000001</v>
       </c>
       <c r="I62">
         <v>134.648</v>
       </c>
       <c r="K62">
-        <v>0.201</v>
+        <v>0.20100000000000001</v>
       </c>
       <c r="L62">
-        <v>0.802</v>
+        <v>0.80200000000000005</v>
       </c>
       <c r="M62">
         <v>0.62</v>
@@ -3728,13 +3678,13 @@
         <v>15608.4</v>
       </c>
       <c r="O62">
-        <v>46.226</v>
+        <v>46.225999999999999</v>
       </c>
       <c r="Q62">
-        <v>0.233</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="R62">
-        <v>0.002</v>
+        <v>2E-3</v>
       </c>
       <c r="S62">
         <v>1.399</v>
@@ -3743,42 +3693,42 @@
         <v>50230.6</v>
       </c>
       <c r="U62">
-        <v>112.118</v>
+        <v>112.11799999999999</v>
       </c>
       <c r="W62">
         <v>0.214</v>
       </c>
       <c r="X62">
-        <v>0.597</v>
-      </c>
-    </row>
-    <row r="63">
+        <v>0.59699999999999998</v>
+      </c>
+    </row>
+    <row r="63" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>2011</v>
       </c>
       <c r="B63">
-        <v>76748.89999999999</v>
+        <v>76748.899999999994</v>
       </c>
       <c r="C63">
         <v>110.822</v>
       </c>
       <c r="E63">
-        <v>0.228</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="F63">
-        <v>0.586</v>
+        <v>0.58599999999999997</v>
       </c>
       <c r="H63">
         <v>8018.3</v>
       </c>
       <c r="I63">
-        <v>142.396</v>
+        <v>142.39599999999999</v>
       </c>
       <c r="K63">
-        <v>0.167</v>
+        <v>0.16700000000000001</v>
       </c>
       <c r="L63">
-        <v>0.916</v>
+        <v>0.91600000000000004</v>
       </c>
       <c r="M63">
         <v>0.6</v>
@@ -3787,45 +3737,45 @@
         <v>17959.7</v>
       </c>
       <c r="O63">
-        <v>52.251</v>
+        <v>52.250999999999998</v>
       </c>
       <c r="Q63">
-        <v>0.334</v>
+        <v>0.33400000000000002</v>
       </c>
       <c r="R63">
-        <v>0.028</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="S63">
-        <v>0.956</v>
+        <v>0.95599999999999996</v>
       </c>
       <c r="T63">
         <v>50770.9</v>
       </c>
       <c r="U63">
-        <v>111.945</v>
+        <v>111.94499999999999</v>
       </c>
       <c r="W63">
-        <v>0.226</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="X63">
-        <v>0.593</v>
-      </c>
-    </row>
-    <row r="64">
+        <v>0.59299999999999997</v>
+      </c>
+    </row>
+    <row r="64" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>2012</v>
       </c>
       <c r="B64">
-        <v>71315.60000000001</v>
+        <v>71315.600000000006</v>
       </c>
       <c r="C64">
-        <v>104.844</v>
+        <v>104.84399999999999</v>
       </c>
       <c r="E64">
-        <v>0.211</v>
+        <v>0.21099999999999999</v>
       </c>
       <c r="F64">
-        <v>0.535</v>
+        <v>0.53500000000000003</v>
       </c>
       <c r="H64">
         <v>7192.4</v>
@@ -3834,28 +3784,28 @@
         <v>134.417</v>
       </c>
       <c r="K64">
-        <v>0.164</v>
+        <v>0.16400000000000001</v>
       </c>
       <c r="L64">
-        <v>0.785</v>
+        <v>0.78500000000000003</v>
       </c>
       <c r="M64">
-        <v>0.631</v>
+        <v>0.63100000000000001</v>
       </c>
       <c r="N64">
         <v>16672.2</v>
       </c>
       <c r="O64">
-        <v>50.642</v>
+        <v>50.642000000000003</v>
       </c>
       <c r="Q64">
-        <v>0.292</v>
+        <v>0.29199999999999998</v>
       </c>
       <c r="R64">
-        <v>0.015</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="S64">
-        <v>0.632</v>
+        <v>0.63200000000000001</v>
       </c>
       <c r="T64">
         <v>47451</v>
@@ -3864,18 +3814,18 @@
         <v>107.083</v>
       </c>
       <c r="W64">
-        <v>0.207</v>
+        <v>0.20699999999999999</v>
       </c>
       <c r="X64">
-        <v>0.5600000000000001</v>
-      </c>
-    </row>
-    <row r="65">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="65" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>2013</v>
       </c>
       <c r="B65">
-        <v>66975.60000000001</v>
+        <v>66975.600000000006</v>
       </c>
       <c r="C65">
         <v>105.685</v>
@@ -3884,66 +3834,66 @@
         <v>0.247</v>
       </c>
       <c r="F65">
-        <v>0.529</v>
+        <v>0.52900000000000003</v>
       </c>
       <c r="H65">
         <v>7740.8</v>
       </c>
       <c r="I65">
-        <v>137.163</v>
+        <v>137.16300000000001</v>
       </c>
       <c r="K65">
-        <v>0.172</v>
+        <v>0.17199999999999999</v>
       </c>
       <c r="L65">
-        <v>0.8120000000000001</v>
+        <v>0.81200000000000006</v>
       </c>
       <c r="M65">
-        <v>0.803</v>
+        <v>0.80300000000000005</v>
       </c>
       <c r="N65">
         <v>16338.5</v>
       </c>
       <c r="O65">
-        <v>49.912</v>
+        <v>49.911999999999999</v>
       </c>
       <c r="Q65">
-        <v>0.333</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="R65">
-        <v>0.018</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="S65">
-        <v>0.661</v>
+        <v>0.66100000000000003</v>
       </c>
       <c r="T65">
         <v>42896.3</v>
       </c>
       <c r="U65">
-        <v>108.055</v>
+        <v>108.05500000000001</v>
       </c>
       <c r="W65">
         <v>0.246</v>
       </c>
       <c r="X65">
-        <v>0.551</v>
-      </c>
-    </row>
-    <row r="66">
+        <v>0.55100000000000005</v>
+      </c>
+    </row>
+    <row r="66" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>2014</v>
       </c>
       <c r="B66">
-        <v>75307.2</v>
+        <v>75307.199999999997</v>
       </c>
       <c r="C66">
-        <v>107.912</v>
+        <v>107.91200000000001</v>
       </c>
       <c r="E66">
-        <v>0.242</v>
+        <v>0.24199999999999999</v>
       </c>
       <c r="F66">
-        <v>0.575</v>
+        <v>0.57499999999999996</v>
       </c>
       <c r="H66">
         <v>9272</v>
@@ -3952,25 +3902,25 @@
         <v>134.297</v>
       </c>
       <c r="K66">
-        <v>0.172</v>
+        <v>0.17199999999999999</v>
       </c>
       <c r="L66">
-        <v>0.881</v>
+        <v>0.88100000000000001</v>
       </c>
       <c r="M66">
-        <v>0.854</v>
+        <v>0.85399999999999998</v>
       </c>
       <c r="N66">
         <v>16892.7</v>
       </c>
       <c r="O66">
-        <v>51.729</v>
+        <v>51.728999999999999</v>
       </c>
       <c r="Q66">
-        <v>0.383</v>
+        <v>0.38300000000000001</v>
       </c>
       <c r="R66">
-        <v>0.042</v>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="S66">
         <v>0.76</v>
@@ -3982,18 +3932,18 @@
         <v>110.75</v>
       </c>
       <c r="W66">
-        <v>0.236</v>
+        <v>0.23599999999999999</v>
       </c>
       <c r="X66">
-        <v>0.597</v>
-      </c>
-    </row>
-    <row r="67">
+        <v>0.59699999999999998</v>
+      </c>
+    </row>
+    <row r="67" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>2015</v>
       </c>
       <c r="B67">
-        <v>79793.60000000001</v>
+        <v>79793.600000000006</v>
       </c>
       <c r="C67">
         <v>107.503</v>
@@ -4002,10 +3952,10 @@
         <v>0.214</v>
       </c>
       <c r="F67">
-        <v>0.5629999999999999</v>
+        <v>0.56299999999999994</v>
       </c>
       <c r="H67">
-        <v>9168.799999999999</v>
+        <v>9168.7999999999993</v>
       </c>
       <c r="I67">
         <v>119.718</v>
@@ -4014,31 +3964,31 @@
         <v>0.16</v>
       </c>
       <c r="L67">
-        <v>0.788</v>
+        <v>0.78800000000000003</v>
       </c>
       <c r="M67">
         <v>0.875</v>
       </c>
       <c r="N67">
-        <v>16648.1</v>
+        <v>16648.099999999999</v>
       </c>
       <c r="O67">
-        <v>49.854</v>
+        <v>49.853999999999999</v>
       </c>
       <c r="Q67">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="R67">
-        <v>0.013</v>
+        <v>1.2999999999999999E-2</v>
       </c>
       <c r="S67">
-        <v>0.765</v>
+        <v>0.76500000000000001</v>
       </c>
       <c r="T67">
         <v>53976.7</v>
       </c>
       <c r="U67">
-        <v>113.076</v>
+        <v>113.07599999999999</v>
       </c>
       <c r="W67">
         <v>0.21</v>
@@ -4047,7 +3997,7 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>2016</v>
       </c>
@@ -4055,13 +4005,13 @@
         <v>79337.2</v>
       </c>
       <c r="C68">
-        <v>97.916</v>
+        <v>97.915999999999997</v>
       </c>
       <c r="E68">
         <v>0.254</v>
       </c>
       <c r="F68">
-        <v>0.423</v>
+        <v>0.42299999999999999</v>
       </c>
       <c r="H68">
         <v>8170.9</v>
@@ -4070,43 +4020,43 @@
         <v>120.77</v>
       </c>
       <c r="K68">
-        <v>0.201</v>
+        <v>0.20100000000000001</v>
       </c>
       <c r="L68">
-        <v>0.6820000000000001</v>
+        <v>0.68200000000000005</v>
       </c>
       <c r="M68">
-        <v>0.803</v>
+        <v>0.80300000000000005</v>
       </c>
       <c r="N68">
         <v>19972.7</v>
       </c>
       <c r="O68">
-        <v>48.868</v>
+        <v>48.868000000000002</v>
       </c>
       <c r="Q68">
-        <v>0.283</v>
+        <v>0.28299999999999997</v>
       </c>
       <c r="R68">
-        <v>0.006</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="S68">
-        <v>0.778</v>
+        <v>0.77800000000000002</v>
       </c>
       <c r="T68">
-        <v>51193.6</v>
+        <v>51193.599999999999</v>
       </c>
       <c r="U68">
-        <v>101.106</v>
+        <v>101.10599999999999</v>
       </c>
       <c r="W68">
         <v>0.255</v>
       </c>
       <c r="X68">
-        <v>0.445</v>
-      </c>
-    </row>
-    <row r="69">
+        <v>0.44500000000000001</v>
+      </c>
+    </row>
+    <row r="69" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>2017</v>
       </c>
@@ -4114,7 +4064,7 @@
         <v>78617.5</v>
       </c>
       <c r="C69">
-        <v>96.27800000000001</v>
+        <v>96.278000000000006</v>
       </c>
       <c r="E69">
         <v>0.254</v>
@@ -4123,31 +4073,31 @@
         <v>0.432</v>
       </c>
       <c r="H69">
-        <v>8512.700000000001</v>
+        <v>8512.7000000000007</v>
       </c>
       <c r="I69">
         <v>126.68</v>
       </c>
       <c r="K69">
-        <v>0.204</v>
+        <v>0.20399999999999999</v>
       </c>
       <c r="L69">
         <v>0.748</v>
       </c>
       <c r="M69">
-        <v>0.773</v>
+        <v>0.77300000000000002</v>
       </c>
       <c r="N69">
         <v>20014.2</v>
       </c>
       <c r="O69">
-        <v>50.635</v>
+        <v>50.634999999999998</v>
       </c>
       <c r="Q69">
-        <v>0.355</v>
+        <v>0.35499999999999998</v>
       </c>
       <c r="R69">
-        <v>0.027</v>
+        <v>2.7E-2</v>
       </c>
       <c r="S69">
         <v>1.022</v>
@@ -4156,7 +4106,7 @@
         <v>50090.6</v>
       </c>
       <c r="U69">
-        <v>97.664</v>
+        <v>97.664000000000001</v>
       </c>
       <c r="W69">
         <v>0.249</v>
@@ -4165,7 +4115,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>2018</v>
       </c>
@@ -4176,55 +4126,55 @@
         <v>105.41</v>
       </c>
       <c r="E70">
-        <v>0.238</v>
+        <v>0.23799999999999999</v>
       </c>
       <c r="F70">
-        <v>0.534</v>
+        <v>0.53400000000000003</v>
       </c>
       <c r="H70">
         <v>6963.8</v>
       </c>
       <c r="I70">
-        <v>132.872</v>
+        <v>132.87200000000001</v>
       </c>
       <c r="K70">
-        <v>0.204</v>
+        <v>0.20399999999999999</v>
       </c>
       <c r="L70">
-        <v>0.833</v>
+        <v>0.83299999999999996</v>
       </c>
       <c r="M70">
-        <v>0.671</v>
+        <v>0.67100000000000004</v>
       </c>
       <c r="N70">
-        <v>19893.6</v>
+        <v>19893.599999999999</v>
       </c>
       <c r="O70">
-        <v>50.398</v>
+        <v>50.398000000000003</v>
       </c>
       <c r="Q70">
         <v>0.31</v>
       </c>
       <c r="R70">
-        <v>0.023</v>
+        <v>2.3E-2</v>
       </c>
       <c r="S70">
-        <v>1.527</v>
+        <v>1.5269999999999999</v>
       </c>
       <c r="T70">
         <v>46113.4</v>
       </c>
       <c r="U70">
-        <v>107.132</v>
+        <v>107.13200000000001</v>
       </c>
       <c r="W70">
-        <v>0.236</v>
+        <v>0.23599999999999999</v>
       </c>
       <c r="X70">
-        <v>0.547</v>
-      </c>
-    </row>
-    <row r="71">
+        <v>0.54700000000000004</v>
+      </c>
+    </row>
+    <row r="71" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>2019</v>
       </c>
@@ -4238,37 +4188,37 @@
         <v>0.224</v>
       </c>
       <c r="F71">
-        <v>0.586</v>
+        <v>0.58599999999999997</v>
       </c>
       <c r="H71">
         <v>7735.3</v>
       </c>
       <c r="I71">
-        <v>129.093</v>
+        <v>129.09299999999999</v>
       </c>
       <c r="K71">
         <v>0.193</v>
       </c>
       <c r="L71">
-        <v>0.789</v>
+        <v>0.78900000000000003</v>
       </c>
       <c r="M71">
-        <v>0.722</v>
+        <v>0.72199999999999998</v>
       </c>
       <c r="N71">
         <v>15302.3</v>
       </c>
       <c r="O71">
-        <v>51.154</v>
+        <v>51.154000000000003</v>
       </c>
       <c r="Q71">
-        <v>0.353</v>
+        <v>0.35299999999999998</v>
       </c>
       <c r="R71">
-        <v>0.025</v>
+        <v>2.5000000000000001E-2</v>
       </c>
       <c r="S71">
-        <v>1.499</v>
+        <v>1.4990000000000001</v>
       </c>
       <c r="T71">
         <v>52607.9</v>
@@ -4280,7 +4230,7 @@
         <v>0.221</v>
       </c>
       <c r="X71">
-        <v>0.597</v>
+        <v>0.59699999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>